<commit_message>
new commmit with latest and working code
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/INPUTS/shared-classes-template.xlsx
+++ b/TIME TABLE SAMPLE DATA/INPUTS/shared-classes-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajas\OneDrive\Desktop\Timetable\TIME TABLE SAMPLE DATA\INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A40659A-2FD4-45ED-A822-E9D84CC41E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CA27F1-DB8D-45F1-9F84-992E43D1B1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>year</t>
   </si>
@@ -29,9 +29,6 @@
   </si>
   <si>
     <t>subject</t>
-  </si>
-  <si>
-    <t>C2,C3</t>
   </si>
 </sst>
 </file>
@@ -394,7 +391,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -408,17 +405,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>